<commit_message>
Suma 8 entidades patrocinantes RM desde la nomina MINVU junio 2026
La descarga de la nomina oficial no fue posible: la politica de red del
entorno rechaza la conexion a los dominios MINVU en el gateway de salida
(403 al CONNECT, en los tres hosts probados). Queda documentado en el
README junto con las URLs para bajarla manualmente.

Via indices de busqueda sobre el PDF se recuperaron 8 entidades
patrocinantes de la Region Metropolitana que no estaban en el
levantamiento: Evolutiva, Kutralwe, Jessica Sandoval Quiroga EIRL,
Manuel Medina EIRL, Gestora Mashogar, Inmobiliaria D&M, Nahuen
Ingenieros Constructores Asociados y Avalos y Ibacache Arquitectos
Sociales. Solo el nombre; RUT, telefono y correo siguen pendientes.

Total: 44 entidades (27 DS19, 26 DS49), 34 con presencia en la RM.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F6LuEua9T1msVfVykNtNcn
</commit_message>
<xml_diff>
--- a/inmobiliarias-santiago/inmobiliarias_ds19_ds49.xlsx
+++ b/inmobiliarias-santiago/inmobiliarias_ds19_ds49.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'DS19'!$A$4:$K$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DS49'!$A$4:$K$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DS49'!$A$4:$K$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2248,7 +2248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2965,12 +2965,12 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Fundación Deportistas por un Sueño</t>
+          <t>Entidad Patrocinante Jessica Sandoval Quiroga E.I.R.L.</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Fundación</t>
+          <t>Entidad Patrocinante</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -3000,12 +3000,12 @@
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>Por confirmar</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>ADVS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J16" s="13" t="inlineStr">
@@ -3015,24 +3015,24 @@
       </c>
       <c r="K16" s="9" t="inlineStr">
         <is>
-          <t>Nómina de socios ADVS</t>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Grupo Vías</t>
+          <t>Entidad Patrocinante Kutralwe Ltda</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Inmobiliaria</t>
+          <t>Entidad Patrocinante</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>DS19 / DS49</t>
+          <t>DS49</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -3057,12 +3057,12 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Por confirmar</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>ADVS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J17" s="13" t="inlineStr">
@@ -3072,19 +3072,19 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Nómina de socios ADVS</t>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Ilustre Municipalidad de Huechuraba</t>
+          <t>Entidad Patrocinante Manuel Medina E.I.R.L.</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Municipio / Entidad Patrocinante</t>
+          <t>Entidad Patrocinante</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -3092,9 +3092,9 @@
           <t>DS49</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>huechuraba.cl</t>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>No identificado</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Huechuraba</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
@@ -3129,19 +3129,19 @@
       </c>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>Nómina MINVU de entidades patrocinantes</t>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Inmobiliaria y Constructora INSOC Ltda</t>
+          <t>Evolutiva Entidad Patrocinante y Consultora de Vivienda y Urbanismo SpA</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Constructora / Entidad Patrocinante</t>
+          <t>Entidad Patrocinante</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Región Metropolitana</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -3186,34 +3186,34 @@
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Nómina MINVU de entidades patrocinantes</t>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>TECHO-Chile (Inmobiliaria Social)</t>
+          <t>Fundación Deportistas por un Sueño</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Fundación / desarrolladora</t>
+          <t>Fundación</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>DS49 colectivo</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>cl.techo.org</t>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>No identificado</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>No publicado (formulario web)</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -3223,12 +3223,12 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Por confirmar</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
@@ -3243,34 +3243,34 @@
       </c>
       <c r="K20" s="9" t="inlineStr">
         <is>
-          <t>Página Inmobiliaria Social</t>
+          <t>Nómina de socios ADVS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Urbanismo Social / Fundación Gestión Vivienda</t>
+          <t>Gestora Mashogar Ltda</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Fundación / Entidad Patrocinante</t>
+          <t>Entidad Patrocinante</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>DS49 / DS19</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>urbanismosocial.cl</t>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>No identificado</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>No publicado (formulario web)</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>No publicado</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>ADVS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J21" s="13" t="inlineStr">
@@ -3300,69 +3300,525 @@
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>Sitio corporativo</t>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
+          <t>Grupo Vías</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Inmobiliaria</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>DS19 / DS49</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>ADVS</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>Nómina de socios ADVS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Ilustre Municipalidad de Huechuraba</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Municipio / Entidad Patrocinante</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>huechuraba.cl</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Huechuraba</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Nómina MINVU de entidades patrocinantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Inmobiliaria D&amp;M SpA</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Entidad Patrocinante / Inmobiliaria</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Inmobiliaria y Constructora INSOC Ltda</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Constructora / Entidad Patrocinante</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Nómina MINVU de entidades patrocinantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Nahuen Ingenieros Constructores Asociados SpA</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Entidad Patrocinante / Constructora</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>TECHO-Chile (Inmobiliaria Social)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Fundación / desarrolladora</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>DS49 colectivo</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>cl.techo.org</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>No publicado (formulario web)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>ADVS</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Página Inmobiliaria Social</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Urbanismo Social / Fundación Gestión Vivienda</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Fundación / Entidad Patrocinante</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>DS49 / DS19</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>urbanismosocial.cl</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>No publicado (formulario web)</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Santiago</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>ADVS</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>Sitio corporativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
           <t>Urbanitas</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Inmobiliaria</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>DS19 / DS49</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>No publicado</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>No publicado</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>No publicado</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Por confirmar</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>ADVS</t>
         </is>
       </c>
-      <c r="J22" s="13" t="inlineStr">
+      <c r="J29" s="13" t="inlineStr">
         <is>
           <t>sin dato</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>Nómina de socios ADVS</t>
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Ávalos y Ibacache Arquitectos Sociales Ltda</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Entidad Patrocinante</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>DS49</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>No publicado</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
+        <is>
+          <t>sin dato</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>Nómina MINVU junio 2026 (vía índice de búsqueda)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K22"/>
+  <autoFilter ref="A4:K30"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -3373,9 +3829,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3427,7 +3883,7 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -3437,7 +3893,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7">

</xml_diff>